<commit_message>
Daily EOD data and reports for 2026-07-28
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20260728.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20260728.xlsx
@@ -731,24 +731,24 @@
         </is>
       </c>
       <c r="B13" s="2" t="n">
-        <v>0</v>
+        <v>0.002</v>
       </c>
       <c r="C13" s="2" t="n">
-        <v>-0.002</v>
+        <v>0</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">
         <v>700000</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>0</v>
+        <v>1400</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>-1400</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -785,24 +785,24 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>-0.1</v>
+        <v>0</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>0.00%</t>
         </is>
       </c>
       <c r="E15" s="3" t="n">
         <v>6000</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>-600</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1598592.37</v>
+        <v>1600592.37</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>-4363.01</v>
+        <v>-2363.01</v>
       </c>
     </row>
   </sheetData>

</xml_diff>